<commit_message>
Column names have been updated to reflect the new naming convention. The cumulative columns and available metrics have been adjusted accordingly. The default selected metrics for the graph have also been updated to "법인 매출" and "법인 영업이익".
</commit_message>
<xml_diff>
--- a/비용 정리_260702.xlsx
+++ b/비용 정리_260702.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bkahn/Library/Mobile Documents/com~apple~CloudDocs/0. 사업/1. 결산/Deployment/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF9E251-E1F0-3F4A-932C-75E7399DDFE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE58809-A86E-2244-A0F8-75258A364B96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{22CEC514-C066-E441-9C92-ED07EE8853CA}"/>
   </bookViews>
@@ -1534,7 +1534,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="159">
   <si>
     <t>수익</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2069,6 +2069,18 @@
   <si>
     <t>Jina</t>
   </si>
+  <si>
+    <t>법인 안병규 입금</t>
+  </si>
+  <si>
+    <t>개인사업자 입금</t>
+  </si>
+  <si>
+    <t>법인으로 송금</t>
+  </si>
+  <si>
+    <t>법인 대출</t>
+  </si>
 </sst>
 </file>
 
@@ -2079,7 +2091,7 @@
     <numFmt numFmtId="165" formatCode="###,##0"/>
     <numFmt numFmtId="166" formatCode="#,###"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2141,12 +2153,6 @@
       <name val="pd"/>
       <family val="2"/>
       <charset val="129"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -3331,13 +3337,11 @@
     <col min="20" max="21" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="14.1640625" style="4" customWidth="1"/>
     <col min="23" max="23" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="26" width="14.1640625" style="4" customWidth="1"/>
-    <col min="27" max="27" width="14.1640625" style="4" hidden="1" customWidth="1"/>
+    <col min="24" max="27" width="14.1640625" style="4" customWidth="1"/>
     <col min="28" max="28" width="13.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="13.1640625" style="4" customWidth="1"/>
     <col min="30" max="30" width="18.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13.1640625" style="4" hidden="1" customWidth="1"/>
-    <col min="32" max="33" width="13.1640625" style="4" customWidth="1"/>
+    <col min="31" max="33" width="13.1640625" style="4" customWidth="1"/>
     <col min="34" max="34" width="12.5" style="4" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="14" style="4" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="13.1640625" style="4" hidden="1" customWidth="1"/>
@@ -3457,13 +3461,13 @@
         <v>2</v>
       </c>
       <c r="AC1" s="4" t="s">
-        <v>81</v>
+        <v>155</v>
       </c>
       <c r="AD1" s="4" t="s">
-        <v>95</v>
+        <v>156</v>
       </c>
       <c r="AE1" s="4" t="s">
-        <v>86</v>
+        <v>158</v>
       </c>
       <c r="AF1" s="4" t="s">
         <v>85</v>
@@ -3544,7 +3548,7 @@
         <v>86</v>
       </c>
       <c r="BF1" s="4" t="s">
-        <v>82</v>
+        <v>157</v>
       </c>
       <c r="BG1" s="4" t="s">
         <v>94</v>
@@ -29990,7 +29994,7 @@
         <v>57</v>
       </c>
       <c r="BY33">
-        <f t="shared" ref="BY32:BY33" si="68">BW33*0.1</f>
+        <f t="shared" ref="BY33" si="68">BW33*0.1</f>
         <v>25.5</v>
       </c>
       <c r="BZ33">
@@ -31392,7 +31396,7 @@
         <v>20</v>
       </c>
       <c r="BY45">
-        <f t="shared" ref="BY45:BY46" si="96">BW45*0.1</f>
+        <f t="shared" ref="BY45" si="96">BW45*0.1</f>
         <v>22</v>
       </c>
       <c r="BZ45">

</xml_diff>

<commit_message>
Debugging the code to ensure that the cumulative columns and available metrics are correctly identified and displayed in the Streamlit app. The changes include adding print statements to output the list of columns in the filtered DataFrame and the available metrics for selection. This will help in verifying that the correct columns are being processed and displayed to the user.
</commit_message>
<xml_diff>
--- a/비용 정리_260702.xlsx
+++ b/비용 정리_260702.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bkahn/Library/Mobile Documents/com~apple~CloudDocs/0. 사업/1. 결산/Deployment/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F453F6-E68C-FD4E-B85F-520FF80FC238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{092CB5B0-3541-5549-8C37-E611FC0635E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{22CEC514-C066-E441-9C92-ED07EE8853CA}"/>
   </bookViews>
@@ -3340,7 +3340,9 @@
     <col min="20" max="21" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="14.1640625" style="4" customWidth="1"/>
     <col min="23" max="23" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="28" width="14.1640625" style="4" customWidth="1"/>
+    <col min="24" max="26" width="14.1640625" style="4" customWidth="1"/>
+    <col min="27" max="27" width="17.1640625" style="4" customWidth="1"/>
+    <col min="28" max="28" width="14.1640625" style="4" customWidth="1"/>
     <col min="29" max="29" width="13.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="13.1640625" style="4" customWidth="1"/>
     <col min="31" max="31" width="18.33203125" style="4" bestFit="1" customWidth="1"/>

</xml_diff>